<commit_message>
Update NBA game results for December 28, 2025 in nba2026.csv and related files
</commit_message>
<xml_diff>
--- a/data/processed/nba/2025-26/report.xlsx
+++ b/data/processed/nba/2025-26/report.xlsx
@@ -496,10 +496,10 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>4.398642315825829</v>
+        <v>4.398642315825834</v>
       </c>
       <c r="C2">
-        <v>9.811197825477377</v>
+        <v>9.811197825477386</v>
       </c>
       <c r="D2">
         <v>31</v>
@@ -510,10 +510,10 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>2.96912861623146</v>
+        <v>2.969128616231461</v>
       </c>
       <c r="C3">
-        <v>7.208024727891347</v>
+        <v>7.208024727891353</v>
       </c>
       <c r="D3">
         <v>31</v>
@@ -527,7 +527,7 @@
         <v>2.324238292750519</v>
       </c>
       <c r="C4">
-        <v>5.586114981917394</v>
+        <v>5.586114981917396</v>
       </c>
       <c r="D4">
         <v>31</v>
@@ -538,10 +538,10 @@
         <v>7</v>
       </c>
       <c r="B5">
-        <v>2.147498360453235</v>
+        <v>2.147498360453234</v>
       </c>
       <c r="C5">
-        <v>5.062279443862951</v>
+        <v>5.06227944386295</v>
       </c>
       <c r="D5">
         <v>30</v>
@@ -552,10 +552,10 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>1.989558265803863</v>
+        <v>1.989558265803864</v>
       </c>
       <c r="C6">
-        <v>4.556312373839581</v>
+        <v>4.556312373839585</v>
       </c>
       <c r="D6">
         <v>31</v>
@@ -569,7 +569,7 @@
         <v>1.686108412130946</v>
       </c>
       <c r="C7">
-        <v>3.460211333292929</v>
+        <v>3.46021133329293</v>
       </c>
       <c r="D7">
         <v>29</v>
@@ -583,7 +583,7 @@
         <v>1.621894633943499</v>
       </c>
       <c r="C8">
-        <v>3.203037321434917</v>
+        <v>3.203037321434918</v>
       </c>
       <c r="D8">
         <v>31</v>
@@ -594,10 +594,10 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>1.615639318007632</v>
+        <v>1.615639318007633</v>
       </c>
       <c r="C9">
-        <v>3.1774428799271</v>
+        <v>3.177442879927102</v>
       </c>
       <c r="D9">
         <v>28</v>
@@ -608,10 +608,10 @@
         <v>12</v>
       </c>
       <c r="B10">
-        <v>1.455204789342308</v>
+        <v>1.455204789342309</v>
       </c>
       <c r="C10">
-        <v>2.484741786854622</v>
+        <v>2.484741786854626</v>
       </c>
       <c r="D10">
         <v>30</v>
@@ -622,10 +622,10 @@
         <v>13</v>
       </c>
       <c r="B11">
-        <v>1.281196794608006</v>
+        <v>1.281196794608007</v>
       </c>
       <c r="C11">
-        <v>1.641240048937576</v>
+        <v>1.641240048937578</v>
       </c>
       <c r="D11">
         <v>30</v>
@@ -636,10 +636,10 @@
         <v>14</v>
       </c>
       <c r="B12">
-        <v>1.206829489424308</v>
+        <v>1.206829489424309</v>
       </c>
       <c r="C12">
-        <v>1.245174867353222</v>
+        <v>1.245174867353225</v>
       </c>
       <c r="D12">
         <v>31</v>
@@ -650,10 +650,10 @@
         <v>15</v>
       </c>
       <c r="B13">
-        <v>0.9707543435401073</v>
+        <v>0.9707543435401075</v>
       </c>
       <c r="C13">
-        <v>-0.1965943190790777</v>
+        <v>-0.1965943190790762</v>
       </c>
       <c r="D13">
         <v>31</v>
@@ -664,10 +664,10 @@
         <v>16</v>
       </c>
       <c r="B14">
-        <v>0.9530049783502417</v>
+        <v>0.9530049783502421</v>
       </c>
       <c r="C14">
-        <v>-0.3188177893880141</v>
+        <v>-0.3188177893880112</v>
       </c>
       <c r="D14">
         <v>31</v>
@@ -681,7 +681,7 @@
         <v>0.8961823568681099</v>
       </c>
       <c r="C15">
-        <v>-0.7259986000295324</v>
+        <v>-0.7259986000295326</v>
       </c>
       <c r="D15">
         <v>29</v>
@@ -692,10 +692,10 @@
         <v>18</v>
       </c>
       <c r="B16">
-        <v>0.8480479191435406</v>
+        <v>0.8480479191435411</v>
       </c>
       <c r="C16">
-        <v>-1.091654482892898</v>
+        <v>-1.091654482892895</v>
       </c>
       <c r="D16">
         <v>32</v>
@@ -706,10 +706,10 @@
         <v>19</v>
       </c>
       <c r="B17">
-        <v>0.78855159714815</v>
+        <v>0.7885515971481505</v>
       </c>
       <c r="C17">
-        <v>-1.573435105216526</v>
+        <v>-1.573435105216523</v>
       </c>
       <c r="D17">
         <v>32</v>
@@ -720,10 +720,10 @@
         <v>20</v>
       </c>
       <c r="B18">
-        <v>0.7657148008854416</v>
+        <v>0.7657148008854417</v>
       </c>
       <c r="C18">
-        <v>-1.768083655575308</v>
+        <v>-1.768083655575307</v>
       </c>
       <c r="D18">
         <v>31</v>
@@ -734,10 +734,10 @@
         <v>21</v>
       </c>
       <c r="B19">
-        <v>0.7101329312629909</v>
+        <v>0.7101329312629912</v>
       </c>
       <c r="C19">
-        <v>-2.267206274440571</v>
+        <v>-2.267206274440569</v>
       </c>
       <c r="D19">
         <v>30</v>
@@ -748,7 +748,7 @@
         <v>22</v>
       </c>
       <c r="B20">
-        <v>0.6998376834979995</v>
+        <v>0.6998376834979996</v>
       </c>
       <c r="C20">
         <v>-2.363932592988374</v>
@@ -762,10 +762,10 @@
         <v>23</v>
       </c>
       <c r="B21">
-        <v>0.60668193277722</v>
+        <v>0.6066819327772202</v>
       </c>
       <c r="C21">
-        <v>-3.310042335345519</v>
+        <v>-3.310042335345518</v>
       </c>
       <c r="D21">
         <v>31</v>
@@ -779,7 +779,7 @@
         <v>0.5663773470493484</v>
       </c>
       <c r="C22">
-        <v>-3.765361242425275</v>
+        <v>-3.765361242425276</v>
       </c>
       <c r="D22">
         <v>30</v>
@@ -790,10 +790,10 @@
         <v>25</v>
       </c>
       <c r="B23">
-        <v>0.4795732021652288</v>
+        <v>0.479573202165229</v>
       </c>
       <c r="C23">
-        <v>-4.867254585145765</v>
+        <v>-4.867254585145763</v>
       </c>
       <c r="D23">
         <v>32</v>
@@ -804,7 +804,7 @@
         <v>26</v>
       </c>
       <c r="B24">
-        <v>0.4424269176600618</v>
+        <v>0.4424269176600619</v>
       </c>
       <c r="C24">
         <v>-5.401240434316214</v>
@@ -821,7 +821,7 @@
         <v>0.4028073732957825</v>
       </c>
       <c r="C25">
-        <v>-6.022625691063181</v>
+        <v>-6.022625691063182</v>
       </c>
       <c r="D25">
         <v>30</v>
@@ -832,10 +832,10 @@
         <v>28</v>
       </c>
       <c r="B26">
-        <v>0.390372659735364</v>
+        <v>0.3903726597353642</v>
       </c>
       <c r="C26">
-        <v>-6.230312921107851</v>
+        <v>-6.23031292110785</v>
       </c>
       <c r="D26">
         <v>31</v>
@@ -860,10 +860,10 @@
         <v>30</v>
       </c>
       <c r="B28">
-        <v>0.3413386628007226</v>
+        <v>0.3413386628007227</v>
       </c>
       <c r="C28">
-        <v>-7.119348383471387</v>
+        <v>-7.119348383471386</v>
       </c>
       <c r="D28">
         <v>30</v>
@@ -874,7 +874,7 @@
         <v>31</v>
       </c>
       <c r="B29">
-        <v>0.3026457903716627</v>
+        <v>0.3026457903716628</v>
       </c>
       <c r="C29">
         <v>-7.916221568168644</v>
@@ -888,7 +888,7 @@
         <v>32</v>
       </c>
       <c r="B30">
-        <v>0.1866519528159469</v>
+        <v>0.186651952815947</v>
       </c>
       <c r="C30">
         <v>-11.11742058314948</v>

</xml_diff>

<commit_message>
Add initial rankings data for NBA teams in rankings-1.csv
</commit_message>
<xml_diff>
--- a/data/processed/nba/2025-26/report.xlsx
+++ b/data/processed/nba/2025-26/report.xlsx
@@ -496,10 +496,10 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>4.398642315825834</v>
+        <v>4.398642315825833</v>
       </c>
       <c r="C2">
-        <v>9.811197825477386</v>
+        <v>9.811197825477382</v>
       </c>
       <c r="D2">
         <v>31</v>
@@ -510,10 +510,10 @@
         <v>5</v>
       </c>
       <c r="B3">
-        <v>2.969128616231461</v>
+        <v>2.96912861623146</v>
       </c>
       <c r="C3">
-        <v>7.208024727891353</v>
+        <v>7.208024727891347</v>
       </c>
       <c r="D3">
         <v>31</v>
@@ -527,7 +527,7 @@
         <v>2.324238292750519</v>
       </c>
       <c r="C4">
-        <v>5.586114981917396</v>
+        <v>5.586114981917393</v>
       </c>
       <c r="D4">
         <v>31</v>
@@ -541,7 +541,7 @@
         <v>2.147498360453234</v>
       </c>
       <c r="C5">
-        <v>5.06227944386295</v>
+        <v>5.062279443862948</v>
       </c>
       <c r="D5">
         <v>30</v>
@@ -552,10 +552,10 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>1.989558265803864</v>
+        <v>1.989558265803863</v>
       </c>
       <c r="C6">
-        <v>4.556312373839585</v>
+        <v>4.556312373839582</v>
       </c>
       <c r="D6">
         <v>31</v>
@@ -569,7 +569,7 @@
         <v>1.686108412130946</v>
       </c>
       <c r="C7">
-        <v>3.46021133329293</v>
+        <v>3.460211333292929</v>
       </c>
       <c r="D7">
         <v>29</v>
@@ -583,7 +583,7 @@
         <v>1.621894633943499</v>
       </c>
       <c r="C8">
-        <v>3.203037321434918</v>
+        <v>3.203037321434917</v>
       </c>
       <c r="D8">
         <v>31</v>
@@ -597,7 +597,7 @@
         <v>1.615639318007633</v>
       </c>
       <c r="C9">
-        <v>3.177442879927102</v>
+        <v>3.177442879927101</v>
       </c>
       <c r="D9">
         <v>28</v>
@@ -608,10 +608,10 @@
         <v>12</v>
       </c>
       <c r="B10">
-        <v>1.455204789342309</v>
+        <v>1.455204789342308</v>
       </c>
       <c r="C10">
-        <v>2.484741786854626</v>
+        <v>2.484741786854622</v>
       </c>
       <c r="D10">
         <v>30</v>
@@ -622,10 +622,10 @@
         <v>13</v>
       </c>
       <c r="B11">
-        <v>1.281196794608007</v>
+        <v>1.281196794608006</v>
       </c>
       <c r="C11">
-        <v>1.641240048937578</v>
+        <v>1.641240048937576</v>
       </c>
       <c r="D11">
         <v>30</v>
@@ -639,7 +639,7 @@
         <v>1.206829489424309</v>
       </c>
       <c r="C12">
-        <v>1.245174867353225</v>
+        <v>1.245174867353223</v>
       </c>
       <c r="D12">
         <v>31</v>
@@ -664,10 +664,10 @@
         <v>16</v>
       </c>
       <c r="B14">
-        <v>0.9530049783502421</v>
+        <v>0.9530049783502419</v>
       </c>
       <c r="C14">
-        <v>-0.3188177893880112</v>
+        <v>-0.3188177893880126</v>
       </c>
       <c r="D14">
         <v>31</v>
@@ -678,10 +678,10 @@
         <v>17</v>
       </c>
       <c r="B15">
-        <v>0.8961823568681099</v>
+        <v>0.8961823568681097</v>
       </c>
       <c r="C15">
-        <v>-0.7259986000295326</v>
+        <v>-0.7259986000295341</v>
       </c>
       <c r="D15">
         <v>29</v>
@@ -692,10 +692,10 @@
         <v>18</v>
       </c>
       <c r="B16">
-        <v>0.8480479191435411</v>
+        <v>0.8480479191435408</v>
       </c>
       <c r="C16">
-        <v>-1.091654482892895</v>
+        <v>-1.091654482892896</v>
       </c>
       <c r="D16">
         <v>32</v>
@@ -709,7 +709,7 @@
         <v>0.7885515971481505</v>
       </c>
       <c r="C17">
-        <v>-1.573435105216523</v>
+        <v>-1.573435105216522</v>
       </c>
       <c r="D17">
         <v>32</v>
@@ -720,10 +720,10 @@
         <v>20</v>
       </c>
       <c r="B18">
-        <v>0.7657148008854417</v>
+        <v>0.7657148008854419</v>
       </c>
       <c r="C18">
-        <v>-1.768083655575307</v>
+        <v>-1.768083655575306</v>
       </c>
       <c r="D18">
         <v>31</v>
@@ -734,10 +734,10 @@
         <v>21</v>
       </c>
       <c r="B19">
-        <v>0.7101329312629912</v>
+        <v>0.7101329312629908</v>
       </c>
       <c r="C19">
-        <v>-2.267206274440569</v>
+        <v>-2.267206274440572</v>
       </c>
       <c r="D19">
         <v>30</v>
@@ -748,10 +748,10 @@
         <v>22</v>
       </c>
       <c r="B20">
-        <v>0.6998376834979996</v>
+        <v>0.6998376834979997</v>
       </c>
       <c r="C20">
-        <v>-2.363932592988374</v>
+        <v>-2.363932592988372</v>
       </c>
       <c r="D20">
         <v>32</v>
@@ -762,10 +762,10 @@
         <v>23</v>
       </c>
       <c r="B21">
-        <v>0.6066819327772202</v>
+        <v>0.60668193277722</v>
       </c>
       <c r="C21">
-        <v>-3.310042335345518</v>
+        <v>-3.310042335345519</v>
       </c>
       <c r="D21">
         <v>31</v>
@@ -779,7 +779,7 @@
         <v>0.5663773470493484</v>
       </c>
       <c r="C22">
-        <v>-3.765361242425276</v>
+        <v>-3.765361242425275</v>
       </c>
       <c r="D22">
         <v>30</v>
@@ -790,10 +790,10 @@
         <v>25</v>
       </c>
       <c r="B23">
-        <v>0.479573202165229</v>
+        <v>0.4795732021652289</v>
       </c>
       <c r="C23">
-        <v>-4.867254585145763</v>
+        <v>-4.867254585145764</v>
       </c>
       <c r="D23">
         <v>32</v>
@@ -804,10 +804,10 @@
         <v>26</v>
       </c>
       <c r="B24">
-        <v>0.4424269176600619</v>
+        <v>0.4424269176600618</v>
       </c>
       <c r="C24">
-        <v>-5.401240434316214</v>
+        <v>-5.401240434316215</v>
       </c>
       <c r="D24">
         <v>31</v>
@@ -821,7 +821,7 @@
         <v>0.4028073732957825</v>
       </c>
       <c r="C25">
-        <v>-6.022625691063182</v>
+        <v>-6.022625691063181</v>
       </c>
       <c r="D25">
         <v>30</v>
@@ -835,7 +835,7 @@
         <v>0.3903726597353642</v>
       </c>
       <c r="C26">
-        <v>-6.23031292110785</v>
+        <v>-6.230312921107848</v>
       </c>
       <c r="D26">
         <v>31</v>
@@ -860,10 +860,10 @@
         <v>30</v>
       </c>
       <c r="B28">
-        <v>0.3413386628007227</v>
+        <v>0.3413386628007226</v>
       </c>
       <c r="C28">
-        <v>-7.119348383471386</v>
+        <v>-7.119348383471387</v>
       </c>
       <c r="D28">
         <v>30</v>
@@ -874,7 +874,7 @@
         <v>31</v>
       </c>
       <c r="B29">
-        <v>0.3026457903716628</v>
+        <v>0.3026457903716627</v>
       </c>
       <c r="C29">
         <v>-7.916221568168644</v>
@@ -888,7 +888,7 @@
         <v>32</v>
       </c>
       <c r="B30">
-        <v>0.186651952815947</v>
+        <v>0.1866519528159469</v>
       </c>
       <c r="C30">
         <v>-11.11742058314948</v>
@@ -905,7 +905,7 @@
         <v>0.1680458040194146</v>
       </c>
       <c r="C31">
-        <v>-11.8129364907264</v>
+        <v>-11.81293649072639</v>
       </c>
       <c r="D31">
         <v>31</v>

</xml_diff>

<commit_message>
Update team rankings and add new rankings dataset
- Modified existing rankings in rankings.csv with updated ratings, points, and games for various teams.
- Introduced a new file rankings-2.csv containing an extended dataset of team rankings with detailed statistics.
</commit_message>
<xml_diff>
--- a/data/processed/nba/2025-26/report.xlsx
+++ b/data/processed/nba/2025-26/report.xlsx
@@ -496,7 +496,7 @@
         <v>4</v>
       </c>
       <c r="B2">
-        <v>4.398642315825833</v>
+        <v>4.398642315825832</v>
       </c>
       <c r="C2">
         <v>9.811197825477382</v>
@@ -527,7 +527,7 @@
         <v>2.324238292750519</v>
       </c>
       <c r="C4">
-        <v>5.586114981917393</v>
+        <v>5.586114981917394</v>
       </c>
       <c r="D4">
         <v>31</v>
@@ -552,10 +552,10 @@
         <v>8</v>
       </c>
       <c r="B6">
-        <v>1.989558265803863</v>
+        <v>1.989558265803862</v>
       </c>
       <c r="C6">
-        <v>4.556312373839582</v>
+        <v>4.556312373839579</v>
       </c>
       <c r="D6">
         <v>31</v>
@@ -583,7 +583,7 @@
         <v>1.621894633943499</v>
       </c>
       <c r="C8">
-        <v>3.203037321434917</v>
+        <v>3.203037321434916</v>
       </c>
       <c r="D8">
         <v>31</v>
@@ -594,10 +594,10 @@
         <v>11</v>
       </c>
       <c r="B9">
-        <v>1.615639318007633</v>
+        <v>1.615639318007632</v>
       </c>
       <c r="C9">
-        <v>3.177442879927101</v>
+        <v>3.177442879927098</v>
       </c>
       <c r="D9">
         <v>28</v>
@@ -608,10 +608,10 @@
         <v>12</v>
       </c>
       <c r="B10">
-        <v>1.455204789342308</v>
+        <v>1.455204789342307</v>
       </c>
       <c r="C10">
-        <v>2.484741786854622</v>
+        <v>2.48474178685462</v>
       </c>
       <c r="D10">
         <v>30</v>
@@ -636,10 +636,10 @@
         <v>14</v>
       </c>
       <c r="B12">
-        <v>1.206829489424309</v>
+        <v>1.206829489424308</v>
       </c>
       <c r="C12">
-        <v>1.245174867353223</v>
+        <v>1.245174867353222</v>
       </c>
       <c r="D12">
         <v>31</v>
@@ -650,10 +650,10 @@
         <v>15</v>
       </c>
       <c r="B13">
-        <v>0.9707543435401075</v>
+        <v>0.970754343540107</v>
       </c>
       <c r="C13">
-        <v>-0.1965943190790762</v>
+        <v>-0.1965943190790792</v>
       </c>
       <c r="D13">
         <v>31</v>
@@ -664,10 +664,10 @@
         <v>16</v>
       </c>
       <c r="B14">
-        <v>0.9530049783502419</v>
+        <v>0.9530049783502416</v>
       </c>
       <c r="C14">
-        <v>-0.3188177893880126</v>
+        <v>-0.318817789388015</v>
       </c>
       <c r="D14">
         <v>31</v>
@@ -678,10 +678,10 @@
         <v>17</v>
       </c>
       <c r="B15">
-        <v>0.8961823568681097</v>
+        <v>0.8961823568681094</v>
       </c>
       <c r="C15">
-        <v>-0.7259986000295341</v>
+        <v>-0.7259986000295358</v>
       </c>
       <c r="D15">
         <v>29</v>
@@ -692,10 +692,10 @@
         <v>18</v>
       </c>
       <c r="B16">
-        <v>0.8480479191435408</v>
+        <v>0.8480479191435406</v>
       </c>
       <c r="C16">
-        <v>-1.091654482892896</v>
+        <v>-1.091654482892898</v>
       </c>
       <c r="D16">
         <v>32</v>
@@ -706,10 +706,10 @@
         <v>19</v>
       </c>
       <c r="B17">
-        <v>0.7885515971481505</v>
+        <v>0.7885515971481499</v>
       </c>
       <c r="C17">
-        <v>-1.573435105216522</v>
+        <v>-1.573435105216527</v>
       </c>
       <c r="D17">
         <v>32</v>
@@ -720,10 +720,10 @@
         <v>20</v>
       </c>
       <c r="B18">
-        <v>0.7657148008854419</v>
+        <v>0.7657148008854413</v>
       </c>
       <c r="C18">
-        <v>-1.768083655575306</v>
+        <v>-1.768083655575311</v>
       </c>
       <c r="D18">
         <v>31</v>
@@ -734,10 +734,10 @@
         <v>21</v>
       </c>
       <c r="B19">
-        <v>0.7101329312629908</v>
+        <v>0.7101329312629905</v>
       </c>
       <c r="C19">
-        <v>-2.267206274440572</v>
+        <v>-2.267206274440575</v>
       </c>
       <c r="D19">
         <v>30</v>
@@ -748,10 +748,10 @@
         <v>22</v>
       </c>
       <c r="B20">
-        <v>0.6998376834979997</v>
+        <v>0.6998376834979992</v>
       </c>
       <c r="C20">
-        <v>-2.363932592988372</v>
+        <v>-2.363932592988376</v>
       </c>
       <c r="D20">
         <v>32</v>
@@ -790,10 +790,10 @@
         <v>25</v>
       </c>
       <c r="B23">
-        <v>0.4795732021652289</v>
+        <v>0.4795732021652288</v>
       </c>
       <c r="C23">
-        <v>-4.867254585145764</v>
+        <v>-4.867254585145765</v>
       </c>
       <c r="D23">
         <v>32</v>
@@ -804,10 +804,10 @@
         <v>26</v>
       </c>
       <c r="B24">
-        <v>0.4424269176600618</v>
+        <v>0.4424269176600616</v>
       </c>
       <c r="C24">
-        <v>-5.401240434316215</v>
+        <v>-5.401240434316216</v>
       </c>
       <c r="D24">
         <v>31</v>
@@ -818,10 +818,10 @@
         <v>27</v>
       </c>
       <c r="B25">
-        <v>0.4028073732957825</v>
+        <v>0.4028073732957823</v>
       </c>
       <c r="C25">
-        <v>-6.022625691063181</v>
+        <v>-6.022625691063183</v>
       </c>
       <c r="D25">
         <v>30</v>
@@ -832,10 +832,10 @@
         <v>28</v>
       </c>
       <c r="B26">
-        <v>0.3903726597353642</v>
+        <v>0.3903726597353639</v>
       </c>
       <c r="C26">
-        <v>-6.230312921107848</v>
+        <v>-6.230312921107852</v>
       </c>
       <c r="D26">
         <v>31</v>
@@ -846,10 +846,10 @@
         <v>29</v>
       </c>
       <c r="B27">
-        <v>0.3526235194780891</v>
+        <v>0.352623519478089</v>
       </c>
       <c r="C27">
-        <v>-6.903917120204219</v>
+        <v>-6.90391712020422</v>
       </c>
       <c r="D27">
         <v>28</v>
@@ -860,10 +860,10 @@
         <v>30</v>
       </c>
       <c r="B28">
-        <v>0.3413386628007226</v>
+        <v>0.3413386628007225</v>
       </c>
       <c r="C28">
-        <v>-7.119348383471387</v>
+        <v>-7.119348383471388</v>
       </c>
       <c r="D28">
         <v>30</v>
@@ -877,7 +877,7 @@
         <v>0.3026457903716627</v>
       </c>
       <c r="C29">
-        <v>-7.916221568168644</v>
+        <v>-7.916221568168646</v>
       </c>
       <c r="D29">
         <v>32</v>
@@ -902,10 +902,10 @@
         <v>33</v>
       </c>
       <c r="B31">
-        <v>0.1680458040194146</v>
+        <v>0.1680458040194145</v>
       </c>
       <c r="C31">
-        <v>-11.81293649072639</v>
+        <v>-11.8129364907264</v>
       </c>
       <c r="D31">
         <v>31</v>

</xml_diff>